<commit_message>
data: publish 2026-09-14 rolling operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-09-14-上海公交运营分析.xlsx
+++ b/data/export/2026-09-14-上海公交运营分析.xlsx
@@ -9052,7 +9052,7 @@
       </c>
       <c r="G115" s="1" t="inlineStr">
         <is>
-          <t>旧轨迹模型发现疑似折返信号，但新规则要求：同向连续3次未采到后启动5分钟定向反向追踪，并确认反向推进≥5站；当前尚未取得该确认</t>
+          <t>旧轨迹模型发现疑似折返信号，但新规则要求：同向下一次主采样未再发现该车后立即启动5分钟定向反向追踪，并确认反向推进≥5站；当前尚未取得该确认</t>
         </is>
       </c>
       <c r="H115" s="1" t="inlineStr"/>
@@ -11430,7 +11430,7 @@
       </c>
       <c r="G147" s="1" t="inlineStr">
         <is>
-          <t>旧轨迹模型发现疑似折返信号，但新规则要求：同向连续3次未采到后启动5分钟定向反向追踪，并确认反向推进≥5站；当前尚未取得该确认</t>
+          <t>旧轨迹模型发现疑似折返信号，但新规则要求：同向下一次主采样未再发现该车后立即启动5分钟定向反向追踪，并确认反向推进≥5站；当前尚未取得该确认</t>
         </is>
       </c>
       <c r="H147" s="1" t="inlineStr"/>
@@ -28096,7 +28096,7 @@
       </c>
       <c r="G44" s="1" t="inlineStr">
         <is>
-          <t>旧轨迹模型发现疑似折返信号，但新规则要求：同向连续3次未采到后启动5分钟定向反向追踪，并确认反向推进≥5站；当前尚未取得该确认</t>
+          <t>旧轨迹模型发现疑似折返信号，但新规则要求：同向下一次主采样未再发现该车后立即启动5分钟定向反向追踪，并确认反向推进≥5站；当前尚未取得该确认</t>
         </is>
       </c>
       <c r="H44" s="1" t="inlineStr"/>
@@ -30474,7 +30474,7 @@
       </c>
       <c r="G76" s="1" t="inlineStr">
         <is>
-          <t>旧轨迹模型发现疑似折返信号，但新规则要求：同向连续3次未采到后启动5分钟定向反向追踪，并确认反向推进≥5站；当前尚未取得该确认</t>
+          <t>旧轨迹模型发现疑似折返信号，但新规则要求：同向下一次主采样未再发现该车后立即启动5分钟定向反向追踪，并确认反向推进≥5站；当前尚未取得该确认</t>
         </is>
       </c>
       <c r="H76" s="1" t="inlineStr"/>

</xml_diff>